<commit_message>
feat(PDG-63): onboard DTI_FAIR_TRADE_PRESS_RELEASES adverse-media source
WordPress REST API source (wp-json/wp/v2/posts, category 23). Uses the post
id as the stable external id. Maps title, body, published/updated dates,
author, publisher, article URL, categories, and featured/body images + PDFs
as attachments; pre-normalization extracts image/PDF URLs from the HTML body
(https image files only, excluding the staging domain).
</commit_message>
<xml_diff>
--- a/data/rules/mediaPreNormalization.xlsx
+++ b/data/rules/mediaPreNormalization.xlsx
@@ -1,83 +1,142 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sheet1" sheetId="1" r:id="Re95bdd044535407e"/>
-  </x:sheets>
-</x:workbook>
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30326"/>
+  <workbookPr/>
+  <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
+    <mc:Choice Requires="x15">
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\cloned repos\python-components\data\rules\"/>
+    </mc:Choice>
+  </mc:AlternateContent>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{FE2744A9-3B4C-4EAB-BCA1-D81D2F4E452D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <bookViews>
+    <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="11500" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+  </bookViews>
+  <sheets>
+    <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
+  </sheets>
+  <calcPr calcId="0"/>
+</workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<x:sst xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main"/>
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="18" uniqueCount="14">
+  <si>
+    <t>source</t>
+  </si>
+  <si>
+    <t>entity_type</t>
+  </si>
+  <si>
+    <t>field</t>
+  </si>
+  <si>
+    <t>normalization_type</t>
+  </si>
+  <si>
+    <t>normalization_rule</t>
+  </si>
+  <si>
+    <t>DTI_FAIR_TRADE_PRESS_RELEASES</t>
+  </si>
+  <si>
+    <t>Media</t>
+  </si>
+  <si>
+    <t>content.rendered</t>
+  </si>
+  <si>
+    <t>regex_extract_all</t>
+  </si>
+  <si>
+    <t>ImageUrls</t>
+  </si>
+  <si>
+    <t>&lt;a[^&gt;]+href="([^"]+\.pdf[^"]*)"</t>
+  </si>
+  <si>
+    <t>PdfUrls</t>
+  </si>
+  <si>
+    <t>target_field</t>
+  </si>
+  <si>
+    <t>&lt;img[^&gt;]+src="(https://(?!fteb-staging\.dti\.gov\.ph)[^"]+\.(?:jpe?g|png|webp|gif)(?:\?[^"]*)?)"</t>
+  </si>
+</sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
-<x:styleSheet xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <x:fonts count="2">
-    <x:font>
-      <x:sz val="11"/>
-      <x:name val="Carlito"/>
-    </x:font>
-    <x:font>
-      <x:b/>
-      <x:sz val="11"/>
-      <x:color rgb="FFFFFFFF"/>
-      <x:name val="Carlito"/>
-    </x:font>
-  </x:fonts>
-  <x:fills count="3">
-    <x:fill>
-      <x:patternFill patternType="none"/>
-    </x:fill>
-    <x:fill>
-      <x:patternFill patternType="gray125"/>
-    </x:fill>
-    <x:fill>
-      <x:patternFill patternType="solid">
-        <x:fgColor rgb="FF1F4E78"/>
-      </x:patternFill>
-    </x:fill>
-  </x:fills>
-  <x:borders count="2">
-    <x:border/>
-    <x:border/>
-  </x:borders>
-  <x:cellStyleXfs count="1">
-    <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
-  </x:cellStyleXfs>
-  <x:cellXfs count="13">
-    <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
-    <x:xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
-    <x:xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
-    <x:xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
-    <x:xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <x:alignment wrapText="1"/>
-    </x:xf>
-    <x:xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <x:alignment horizontal="center" wrapText="1"/>
-    </x:xf>
-    <x:xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <x:alignment horizontal="center" vertical="center" wrapText="1"/>
-    </x:xf>
-    <x:xf numFmtId="0" fontId="0" fillId="2" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
-    <x:xf numFmtId="0" fontId="1" fillId="2" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
-    <x:xf numFmtId="0" fontId="1" fillId="2" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <x:alignment wrapText="1"/>
-    </x:xf>
-    <x:xf numFmtId="0" fontId="1" fillId="2" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <x:alignment horizontal="center" wrapText="1"/>
-    </x:xf>
-    <x:xf numFmtId="0" fontId="1" fillId="2" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <x:alignment horizontal="center" vertical="center" wrapText="1"/>
-    </x:xf>
-    <x:xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <x:alignment horizontal="center" vertical="top" wrapText="1"/>
-    </x:xf>
-  </x:cellXfs>
-  <x:cellStyles count="1">
-    <x:cellStyle name="Normal" xfId="0"/>
-  </x:cellStyles>
-</x:styleSheet>
+<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
+  <fonts count="3">
+    <font>
+      <sz val="11"/>
+      <name val="Carlito"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="11"/>
+      <color rgb="FFFFFFFF"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+  </fonts>
+  <fills count="3">
+    <fill>
+      <patternFill patternType="none"/>
+    </fill>
+    <fill>
+      <patternFill patternType="gray125"/>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FF1F4E78"/>
+      </patternFill>
+    </fill>
+  </fills>
+  <borders count="1">
+    <border>
+      <left/>
+      <right/>
+      <top/>
+      <bottom/>
+      <diagonal/>
+    </border>
+  </borders>
+  <cellStyleXfs count="1">
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
+  </cellStyleXfs>
+  <cellXfs count="4">
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
+  </cellXfs>
+  <cellStyles count="1">
+    <cellStyle name="Normal" xfId="0" builtinId="0"/>
+  </cellStyles>
+  <dxfs count="0"/>
+  <tableStyles count="0" defaultTableStyle="TableStyleMedium2" defaultPivotStyle="PivotStyleLight16"/>
+  <extLst>
+    <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{EB79DEF2-80B8-43e5-95BD-54CBDDF9020C}">
+      <x14:slicerStyles defaultSlicerStyle="SlicerStyleLight1"/>
+    </ext>
+    <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{9260A510-F301-46a8-8635-F512D64BE5F5}">
+      <x15:timelineStyles defaultTimelineStyle="TimeSlicerStyleLight1"/>
+    </ext>
+  </extLst>
+</styleSheet>
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
@@ -268,38 +327,85 @@
       </a:bgFillStyleLst>
     </a:fmtScheme>
   </a:themeElements>
+  <a:objectDefaults/>
+  <a:extraClrSchemeLst/>
 </a:theme>
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<x:worksheet xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <x:sheetFormatPr defaultRowHeight="15"/>
-  <x:cols>
-    <x:col min="1" max="1" width="26" hidden="0" customWidth="1"/>
-    <x:col min="2" max="2" width="18" hidden="0" customWidth="1"/>
-    <x:col min="3" max="3" width="34" hidden="0" customWidth="1"/>
-    <x:col min="4" max="4" width="26" hidden="0" customWidth="1"/>
-    <x:col min="5" max="5" width="50" hidden="0" customWidth="1"/>
-  </x:cols>
-  <x:sheetData>
-    <x:row r="1" ht="24" customHeight="1">
-      <x:c r="A1" s="12" t="str">
-        <x:v>source</x:v>
-      </x:c>
-      <x:c r="B1" s="12" t="str">
-        <x:v>entity_type</x:v>
-      </x:c>
-      <x:c r="C1" s="12" t="str">
-        <x:v>field</x:v>
-      </x:c>
-      <x:c r="D1" s="12" t="str">
-        <x:v>normalization_type</x:v>
-      </x:c>
-      <x:c r="E1" s="12" t="str">
-        <x:v>normalization_rule</x:v>
-      </x:c>
-    </x:row>
-  </x:sheetData>
-  <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-</x:worksheet>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
+  <dimension ref="A1:F3"/>
+  <sheetFormatPr defaultRowHeight="14.5"/>
+  <cols>
+    <col min="1" max="1" width="29.6640625" style="2" customWidth="1"/>
+    <col min="2" max="2" width="18" style="2" customWidth="1"/>
+    <col min="3" max="3" width="34" style="2" customWidth="1"/>
+    <col min="4" max="4" width="26" style="2" customWidth="1"/>
+    <col min="5" max="5" width="50" style="2" customWidth="1"/>
+    <col min="6" max="6" width="10.5" style="2" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:6" ht="16" customHeight="1">
+      <c r="A1" s="1" t="s">
+        <v>0</v>
+      </c>
+      <c r="B1" s="1" t="s">
+        <v>1</v>
+      </c>
+      <c r="C1" s="1" t="s">
+        <v>2</v>
+      </c>
+      <c r="D1" s="1" t="s">
+        <v>3</v>
+      </c>
+      <c r="E1" s="1" t="s">
+        <v>4</v>
+      </c>
+      <c r="F1" s="1" t="s">
+        <v>12</v>
+      </c>
+    </row>
+    <row r="2" spans="1:6" ht="28.5">
+      <c r="A2" s="2" t="s">
+        <v>5</v>
+      </c>
+      <c r="B2" s="2" t="s">
+        <v>6</v>
+      </c>
+      <c r="C2" s="2" t="s">
+        <v>7</v>
+      </c>
+      <c r="D2" s="2" t="s">
+        <v>8</v>
+      </c>
+      <c r="E2" s="3" t="s">
+        <v>13</v>
+      </c>
+      <c r="F2" s="2" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="3" spans="1:6">
+      <c r="A3" s="2" t="s">
+        <v>5</v>
+      </c>
+      <c r="B3" s="2" t="s">
+        <v>6</v>
+      </c>
+      <c r="C3" s="2" t="s">
+        <v>7</v>
+      </c>
+      <c r="D3" s="2" t="s">
+        <v>8</v>
+      </c>
+      <c r="E3" s="2" t="s">
+        <v>10</v>
+      </c>
+      <c r="F3" s="2" t="s">
+        <v>11</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
 </file>
</xml_diff>

<commit_message>
feat(PDG-78): onboard DTI_PH_FAIR_TRADE_UPDATES media source
</commit_message>
<xml_diff>
--- a/data/rules/mediaPreNormalization.xlsx
+++ b/data/rules/mediaPreNormalization.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\cloned repos\python-components\data\rules\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{1FFE35B0-3823-4BEF-90AD-B37CA5458313}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A867B548-68A5-42D5-8EAD-7394535CD8F7}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="11500" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -20,7 +20,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="42" uniqueCount="25">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="54" uniqueCount="26">
   <si>
     <t>source</t>
   </si>
@@ -95,6 +95,9 @@
   </si>
   <si>
     <t>&lt;(?:em|i)&gt;(?:&lt;(?:strong|b)&gt;)?\s*By\s+([^&lt;|/]+?)\s*(?:[|/]|&lt;/)</t>
+  </si>
+  <si>
+    <t>DTI_PH_FAIR_TRADE_UPDATES</t>
   </si>
 </sst>
 </file>
@@ -367,7 +370,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:F7"/>
+  <dimension ref="A1:F9"/>
   <sheetFormatPr defaultRowHeight="14.5"/>
   <cols>
     <col min="1" max="1" width="29.6640625" style="2" customWidth="1"/>
@@ -438,29 +441,29 @@
         <v>10</v>
       </c>
     </row>
-    <row r="4" spans="1:6">
+    <row r="4" spans="1:6" ht="27.5" customHeight="1">
       <c r="A4" s="2" t="s">
-        <v>14</v>
+        <v>25</v>
       </c>
       <c r="B4" s="2" t="s">
         <v>5</v>
       </c>
       <c r="C4" s="2" t="s">
-        <v>15</v>
+        <v>6</v>
       </c>
       <c r="D4" s="2" t="s">
         <v>7</v>
       </c>
-      <c r="E4" t="s">
-        <v>17</v>
+      <c r="E4" s="3" t="s">
+        <v>12</v>
       </c>
       <c r="F4" s="2" t="s">
-        <v>16</v>
+        <v>8</v>
       </c>
     </row>
     <row r="5" spans="1:6">
       <c r="A5" s="2" t="s">
-        <v>18</v>
+        <v>25</v>
       </c>
       <c r="B5" s="2" t="s">
         <v>5</v>
@@ -469,33 +472,33 @@
         <v>6</v>
       </c>
       <c r="D5" s="2" t="s">
-        <v>19</v>
+        <v>7</v>
       </c>
       <c r="E5" s="2" t="s">
-        <v>24</v>
-      </c>
-      <c r="F5" t="s">
-        <v>20</v>
+        <v>9</v>
+      </c>
+      <c r="F5" s="2" t="s">
+        <v>10</v>
       </c>
     </row>
     <row r="6" spans="1:6">
       <c r="A6" s="2" t="s">
-        <v>18</v>
+        <v>14</v>
       </c>
       <c r="B6" s="2" t="s">
         <v>5</v>
       </c>
       <c r="C6" s="2" t="s">
-        <v>6</v>
+        <v>15</v>
       </c>
       <c r="D6" s="2" t="s">
         <v>7</v>
       </c>
-      <c r="E6" s="2" t="s">
-        <v>21</v>
+      <c r="E6" t="s">
+        <v>17</v>
       </c>
       <c r="F6" s="2" t="s">
-        <v>8</v>
+        <v>16</v>
       </c>
     </row>
     <row r="7" spans="1:6">
@@ -509,12 +512,52 @@
         <v>6</v>
       </c>
       <c r="D7" s="2" t="s">
-        <v>7</v>
+        <v>19</v>
       </c>
       <c r="E7" s="2" t="s">
+        <v>24</v>
+      </c>
+      <c r="F7" t="s">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="8" spans="1:6">
+      <c r="A8" s="2" t="s">
+        <v>18</v>
+      </c>
+      <c r="B8" s="2" t="s">
+        <v>5</v>
+      </c>
+      <c r="C8" s="2" t="s">
+        <v>6</v>
+      </c>
+      <c r="D8" s="2" t="s">
+        <v>7</v>
+      </c>
+      <c r="E8" s="2" t="s">
+        <v>21</v>
+      </c>
+      <c r="F8" s="2" t="s">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="9" spans="1:6">
+      <c r="A9" s="2" t="s">
+        <v>18</v>
+      </c>
+      <c r="B9" s="2" t="s">
+        <v>5</v>
+      </c>
+      <c r="C9" s="2" t="s">
+        <v>6</v>
+      </c>
+      <c r="D9" s="2" t="s">
+        <v>7</v>
+      </c>
+      <c r="E9" s="2" t="s">
         <v>22</v>
       </c>
-      <c r="F7" s="2" t="s">
+      <c r="F9" s="2" t="s">
         <v>23</v>
       </c>
     </row>

</xml_diff>

<commit_message>
feat(PDG-88): integrate INTERAKSYON_POLITICS_ISSUES and split WordPress categories/tags
Add INTERAKSYON_POLITICS_ISSUES (WordPress REST API, category 15735) with mapping and pre-normalization rules: categories and tags split from wp:term, YouTube embeds as Video attachments, embedded social posts as Related URLs, tracking-pixel gifs excluded. Apply the same category/tag split to PTV_NEWS. Image and document regexes for PTV, DTI and Interaksyon are now case-insensitive and require http(s) links.
</commit_message>
<xml_diff>
--- a/data/rules/mediaPreNormalization.xlsx
+++ b/data/rules/mediaPreNormalization.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30326"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30430"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\cloned repos\python-components\data\rules\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A867B548-68A5-42D5-8EAD-7394535CD8F7}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{C1528568-553E-4FCA-911F-2E75B2E14884}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="11500" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -20,7 +20,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="54" uniqueCount="26">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="102" uniqueCount="37">
   <si>
     <t>source</t>
   </si>
@@ -49,18 +49,12 @@
     <t>ImageUrls</t>
   </si>
   <si>
-    <t>&lt;a[^&gt;]+href="([^"]+\.pdf[^"]*)"</t>
-  </si>
-  <si>
     <t>PdfUrls</t>
   </si>
   <si>
     <t>target_field</t>
   </si>
   <si>
-    <t>&lt;img[^&gt;]+src="(https://(?!fteb-staging\.dti\.gov\.ph)[^"]+\.(?:jpe?g|png|webp|gif)(?:\?[^"]*)?)"</t>
-  </si>
-  <si>
     <t>DTI_PH_FAIR_TRADE_PRESS_RELEASES</t>
   </si>
   <si>
@@ -85,12 +79,6 @@
     <t>Author</t>
   </si>
   <si>
-    <t>&lt;img[^&gt;]+src="([^"]+\.(?:jpe?g|png|webp|gif)(?:\?[^"]*)?)"</t>
-  </si>
-  <si>
-    <t>(?i)&lt;a[^&gt;]+href="([^"]+\.(?:pdf|docx?|xlsx?|pptx?)(?:\?[^"]*)?)"</t>
-  </si>
-  <si>
     <t>DocumentUrls</t>
   </si>
   <si>
@@ -98,6 +86,51 @@
   </si>
   <si>
     <t>DTI_PH_FAIR_TRADE_UPDATES</t>
+  </si>
+  <si>
+    <t>INTERAKSYON_POLITICS_ISSUES</t>
+  </si>
+  <si>
+    <t>_embedded.wp:term</t>
+  </si>
+  <si>
+    <t>WpCategories</t>
+  </si>
+  <si>
+    <t>WpTags</t>
+  </si>
+  <si>
+    <t>(?&lt;='name': ')(?:[^'\\]|\\.)*(?=', 'slug': '(?:[^'\\]|\\.)*', 'taxonomy': 'category')|(?&lt;='name': ")(?:[^"\\]|\\.)*(?=", 'slug': '(?:[^'\\]|\\.)*', 'taxonomy': 'category')</t>
+  </si>
+  <si>
+    <t>(?&lt;='name': ')(?:[^'\\]|\\.)*(?=', 'slug': '(?:[^'\\]|\\.)*', 'taxonomy': 'post_tag')|(?&lt;='name': ")(?:[^"\\]|\\.)*(?=", 'slug': '(?:[^'\\]|\\.)*', 'taxonomy': 'post_tag')</t>
+  </si>
+  <si>
+    <t>VideoUrls</t>
+  </si>
+  <si>
+    <t>SocialUrls</t>
+  </si>
+  <si>
+    <t>(?i)&lt;iframe[^&gt;]+src="(https?://(?:www\.)?youtube(?:-nocookie)?\.com/embed/[\w-]+)</t>
+  </si>
+  <si>
+    <t>https://(?:x|twitter)\.com/\w+/status/\d+|(?&lt;=data-instgrm-permalink=")https://www\.instagram\.com/(?:p|reel)/[\w-]+/|https://www\.facebook\.com/plugins/(?:post|video)\.php\?href=[^"&amp;]+|https://www\.redditmedia\.com/r/[^"?]+</t>
+  </si>
+  <si>
+    <t>(?i)&lt;img[^&gt;]+src="(https://(?!fteb-staging\.dti\.gov\.ph)[^"]+\.(?:jpe?g|png|webp|gif)(?:\?[^"]*)?)"</t>
+  </si>
+  <si>
+    <t>(?i)&lt;a[^&gt;]+href="(https?://[^"]+\.pdf[^"]*)"</t>
+  </si>
+  <si>
+    <t>(?i)&lt;img[^&gt;]+src="(https?://[^"]+\.(?:jpe?g|png|webp|gif)(?:\?[^"]*)?)"</t>
+  </si>
+  <si>
+    <t>(?i)&lt;a[^&gt;]+href="(https?://[^"]+\.(?:pdf|docx?|xlsx?|pptx?)(?:\?[^"]*)?)"</t>
+  </si>
+  <si>
+    <t>(?i)&lt;img[^&gt;]+src="(https?://[^"]+\.(?:jpe?g|png|webp)(?:\?[^"]*)?)"</t>
   </si>
 </sst>
 </file>
@@ -370,7 +403,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:F9"/>
+  <dimension ref="A1:F17"/>
   <sheetFormatPr defaultRowHeight="14.5"/>
   <cols>
     <col min="1" max="1" width="29.6640625" style="2" customWidth="1"/>
@@ -398,12 +431,12 @@
         <v>4</v>
       </c>
       <c r="F1" s="1" t="s">
-        <v>11</v>
+        <v>10</v>
       </c>
     </row>
     <row r="2" spans="1:6" ht="29.5" customHeight="1">
       <c r="A2" s="2" t="s">
-        <v>13</v>
+        <v>11</v>
       </c>
       <c r="B2" s="2" t="s">
         <v>5</v>
@@ -415,7 +448,7 @@
         <v>7</v>
       </c>
       <c r="E2" s="3" t="s">
-        <v>12</v>
+        <v>32</v>
       </c>
       <c r="F2" s="2" t="s">
         <v>8</v>
@@ -423,7 +456,7 @@
     </row>
     <row r="3" spans="1:6">
       <c r="A3" s="2" t="s">
-        <v>13</v>
+        <v>11</v>
       </c>
       <c r="B3" s="2" t="s">
         <v>5</v>
@@ -435,15 +468,15 @@
         <v>7</v>
       </c>
       <c r="E3" s="2" t="s">
+        <v>33</v>
+      </c>
+      <c r="F3" s="2" t="s">
         <v>9</v>
-      </c>
-      <c r="F3" s="2" t="s">
-        <v>10</v>
       </c>
     </row>
     <row r="4" spans="1:6" ht="27.5" customHeight="1">
       <c r="A4" s="2" t="s">
-        <v>25</v>
+        <v>21</v>
       </c>
       <c r="B4" s="2" t="s">
         <v>5</v>
@@ -455,7 +488,7 @@
         <v>7</v>
       </c>
       <c r="E4" s="3" t="s">
-        <v>12</v>
+        <v>32</v>
       </c>
       <c r="F4" s="2" t="s">
         <v>8</v>
@@ -463,7 +496,7 @@
     </row>
     <row r="5" spans="1:6">
       <c r="A5" s="2" t="s">
-        <v>25</v>
+        <v>21</v>
       </c>
       <c r="B5" s="2" t="s">
         <v>5</v>
@@ -475,55 +508,55 @@
         <v>7</v>
       </c>
       <c r="E5" s="2" t="s">
+        <v>33</v>
+      </c>
+      <c r="F5" s="2" t="s">
         <v>9</v>
-      </c>
-      <c r="F5" s="2" t="s">
-        <v>10</v>
       </c>
     </row>
     <row r="6" spans="1:6">
       <c r="A6" s="2" t="s">
+        <v>12</v>
+      </c>
+      <c r="B6" s="2" t="s">
+        <v>5</v>
+      </c>
+      <c r="C6" s="2" t="s">
+        <v>13</v>
+      </c>
+      <c r="D6" s="2" t="s">
+        <v>7</v>
+      </c>
+      <c r="E6" t="s">
+        <v>15</v>
+      </c>
+      <c r="F6" s="2" t="s">
         <v>14</v>
-      </c>
-      <c r="B6" s="2" t="s">
-        <v>5</v>
-      </c>
-      <c r="C6" s="2" t="s">
-        <v>15</v>
-      </c>
-      <c r="D6" s="2" t="s">
-        <v>7</v>
-      </c>
-      <c r="E6" t="s">
-        <v>17</v>
-      </c>
-      <c r="F6" s="2" t="s">
-        <v>16</v>
       </c>
     </row>
     <row r="7" spans="1:6">
       <c r="A7" s="2" t="s">
+        <v>16</v>
+      </c>
+      <c r="B7" s="2" t="s">
+        <v>5</v>
+      </c>
+      <c r="C7" s="2" t="s">
+        <v>6</v>
+      </c>
+      <c r="D7" s="2" t="s">
+        <v>17</v>
+      </c>
+      <c r="E7" s="2" t="s">
+        <v>20</v>
+      </c>
+      <c r="F7" t="s">
         <v>18</v>
-      </c>
-      <c r="B7" s="2" t="s">
-        <v>5</v>
-      </c>
-      <c r="C7" s="2" t="s">
-        <v>6</v>
-      </c>
-      <c r="D7" s="2" t="s">
-        <v>19</v>
-      </c>
-      <c r="E7" s="2" t="s">
-        <v>24</v>
-      </c>
-      <c r="F7" t="s">
-        <v>20</v>
       </c>
     </row>
     <row r="8" spans="1:6">
       <c r="A8" s="2" t="s">
-        <v>18</v>
+        <v>16</v>
       </c>
       <c r="B8" s="2" t="s">
         <v>5</v>
@@ -535,7 +568,7 @@
         <v>7</v>
       </c>
       <c r="E8" s="2" t="s">
-        <v>21</v>
+        <v>34</v>
       </c>
       <c r="F8" s="2" t="s">
         <v>8</v>
@@ -543,7 +576,7 @@
     </row>
     <row r="9" spans="1:6">
       <c r="A9" s="2" t="s">
-        <v>18</v>
+        <v>16</v>
       </c>
       <c r="B9" s="2" t="s">
         <v>5</v>
@@ -555,10 +588,170 @@
         <v>7</v>
       </c>
       <c r="E9" s="2" t="s">
+        <v>35</v>
+      </c>
+      <c r="F9" s="2" t="s">
+        <v>19</v>
+      </c>
+    </row>
+    <row r="10" spans="1:6">
+      <c r="A10" s="2" t="s">
+        <v>16</v>
+      </c>
+      <c r="B10" s="2" t="s">
+        <v>5</v>
+      </c>
+      <c r="C10" s="2" t="s">
+        <v>23</v>
+      </c>
+      <c r="D10" s="2" t="s">
+        <v>7</v>
+      </c>
+      <c r="E10" s="2" t="s">
+        <v>26</v>
+      </c>
+      <c r="F10" s="2" t="s">
+        <v>24</v>
+      </c>
+    </row>
+    <row r="11" spans="1:6">
+      <c r="A11" s="2" t="s">
+        <v>16</v>
+      </c>
+      <c r="B11" s="2" t="s">
+        <v>5</v>
+      </c>
+      <c r="C11" s="2" t="s">
+        <v>23</v>
+      </c>
+      <c r="D11" s="2" t="s">
+        <v>7</v>
+      </c>
+      <c r="E11" s="2" t="s">
+        <v>27</v>
+      </c>
+      <c r="F11" s="2" t="s">
+        <v>25</v>
+      </c>
+    </row>
+    <row r="12" spans="1:6">
+      <c r="A12" s="2" t="s">
         <v>22</v>
       </c>
-      <c r="F9" s="2" t="s">
+      <c r="B12" s="2" t="s">
+        <v>5</v>
+      </c>
+      <c r="C12" s="2" t="s">
+        <v>6</v>
+      </c>
+      <c r="D12" s="2" t="s">
+        <v>7</v>
+      </c>
+      <c r="E12" s="2" t="s">
+        <v>36</v>
+      </c>
+      <c r="F12" s="2" t="s">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="13" spans="1:6">
+      <c r="A13" s="2" t="s">
+        <v>22</v>
+      </c>
+      <c r="B13" s="2" t="s">
+        <v>5</v>
+      </c>
+      <c r="C13" s="2" t="s">
+        <v>6</v>
+      </c>
+      <c r="D13" s="2" t="s">
+        <v>7</v>
+      </c>
+      <c r="E13" s="2" t="s">
+        <v>35</v>
+      </c>
+      <c r="F13" s="2" t="s">
+        <v>19</v>
+      </c>
+    </row>
+    <row r="14" spans="1:6">
+      <c r="A14" s="2" t="s">
+        <v>22</v>
+      </c>
+      <c r="B14" s="2" t="s">
+        <v>5</v>
+      </c>
+      <c r="C14" s="2" t="s">
         <v>23</v>
+      </c>
+      <c r="D14" s="2" t="s">
+        <v>7</v>
+      </c>
+      <c r="E14" s="2" t="s">
+        <v>26</v>
+      </c>
+      <c r="F14" s="2" t="s">
+        <v>24</v>
+      </c>
+    </row>
+    <row r="15" spans="1:6">
+      <c r="A15" s="2" t="s">
+        <v>22</v>
+      </c>
+      <c r="B15" s="2" t="s">
+        <v>5</v>
+      </c>
+      <c r="C15" s="2" t="s">
+        <v>23</v>
+      </c>
+      <c r="D15" s="2" t="s">
+        <v>7</v>
+      </c>
+      <c r="E15" s="2" t="s">
+        <v>27</v>
+      </c>
+      <c r="F15" s="2" t="s">
+        <v>25</v>
+      </c>
+    </row>
+    <row r="16" spans="1:6">
+      <c r="A16" s="2" t="s">
+        <v>22</v>
+      </c>
+      <c r="B16" s="2" t="s">
+        <v>5</v>
+      </c>
+      <c r="C16" s="2" t="s">
+        <v>6</v>
+      </c>
+      <c r="D16" s="2" t="s">
+        <v>7</v>
+      </c>
+      <c r="E16" s="2" t="s">
+        <v>30</v>
+      </c>
+      <c r="F16" s="2" t="s">
+        <v>28</v>
+      </c>
+    </row>
+    <row r="17" spans="1:6">
+      <c r="A17" s="2" t="s">
+        <v>22</v>
+      </c>
+      <c r="B17" s="2" t="s">
+        <v>5</v>
+      </c>
+      <c r="C17" s="2" t="s">
+        <v>6</v>
+      </c>
+      <c r="D17" s="2" t="s">
+        <v>7</v>
+      </c>
+      <c r="E17" s="2" t="s">
+        <v>31</v>
+      </c>
+      <c r="F17" s="2" t="s">
+        <v>29</v>
       </c>
     </row>
   </sheetData>

</xml_diff>